<commit_message>
Adding requirements to the Excel documents to round out the system design.
</commit_message>
<xml_diff>
--- a/examples/GalacticSoup/requirements/SystemRequirements.xlsx
+++ b/examples/GalacticSoup/requirements/SystemRequirements.xlsx
@@ -1,19 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MATLAB_Projects\Playground\galacticSoupKitchen\matlab-mbse-skills\examples\GalacticSoup\requirements\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85FDA84-7020-4B9E-AEF8-0B700E395AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="744" yWindow="1608" windowWidth="21492" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="85" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="128">
   <si>
     <t>Id</t>
   </si>
@@ -244,16 +264,179 @@
   </si>
   <si>
     <t>SN-GS-008</t>
+  </si>
+  <si>
+    <t>SR-GS-017</t>
+  </si>
+  <si>
+    <t>SR-GS-018</t>
+  </si>
+  <si>
+    <t>SR-GS-019</t>
+  </si>
+  <si>
+    <t>SR-GS-020</t>
+  </si>
+  <si>
+    <t>SR-GS-021</t>
+  </si>
+  <si>
+    <t>SR-GS-022</t>
+  </si>
+  <si>
+    <t>SR-GS-023</t>
+  </si>
+  <si>
+    <t>SR-GS-024</t>
+  </si>
+  <si>
+    <t>Concurrent rocket support</t>
+  </si>
+  <si>
+    <t>System shall support simultaneous handling of at least 3 delivery rockets for loading or unloading.</t>
+  </si>
+  <si>
+    <t>Parallel handling prevents outbound shipping from blocking inbound ingredient deliveries.</t>
+  </si>
+  <si>
+    <t>SN-GS-009</t>
+  </si>
+  <si>
+    <t>SN-GS-010</t>
+  </si>
+  <si>
+    <t>SN-GS-011</t>
+  </si>
+  <si>
+    <t>SN-GS-012</t>
+  </si>
+  <si>
+    <t>Rocket turnaround</t>
+  </si>
+  <si>
+    <t>System shall complete loading or unloading of a delivery rocket within 20 minutes.</t>
+  </si>
+  <si>
+    <t>Fast turnaround maximizes fleet utilization and maintains alignment with production throughput.</t>
+  </si>
+  <si>
+    <t>Rocket refueling</t>
+  </si>
+  <si>
+    <t>System shall provide on-site refueling capability for supported delivery rockets.</t>
+  </si>
+  <si>
+    <t>On-site refueling minimizes logistics dependencies and enables rapid redeployment.</t>
+  </si>
+  <si>
+    <t>Temperature-controlled storage</t>
+  </si>
+  <si>
+    <t>System shall provide separate storage zones for cold and room-temperature ingredients.</t>
+  </si>
+  <si>
+    <t>Different ingredient classes require different storage conditions to maintain safety and quality.</t>
+  </si>
+  <si>
+    <t>Ingredient storage capacity</t>
+  </si>
+  <si>
+    <t>System shall store at least 72 hours of ingredients at nominal production rate.</t>
+  </si>
+  <si>
+    <t>72 hours of buffer mitigates delivery delays without exceeding storage mass and volume budgets.</t>
+  </si>
+  <si>
+    <t>Cooking capacity</t>
+  </si>
+  <si>
+    <t>System shall cook soup at a sustained rate sufficient to meet overall throughput requirements.</t>
+  </si>
+  <si>
+    <t>Cooking must not be the bottleneck in achieving 200 bowls/hour system throughput.</t>
+  </si>
+  <si>
+    <t>Internal transfer time</t>
+  </si>
+  <si>
+    <t>Internal transport automation</t>
+  </si>
+  <si>
+    <t>Internal material transport shall be automated for at least 90% of transfers.</t>
+  </si>
+  <si>
+    <t>System shall transport ingredients from storage to cooking at a rate sufficient to sustain nominal cooking throughput.</t>
+  </si>
+  <si>
+    <t>SR-GS-025</t>
+  </si>
+  <si>
+    <t>SR-GS-026</t>
+  </si>
+  <si>
+    <t>SR-GS-027</t>
+  </si>
+  <si>
+    <t>Startup readiness</t>
+  </si>
+  <si>
+    <t>System shall reach nominal operating throughput within a defined startup period after activation.</t>
+  </si>
+  <si>
+    <t>SN-GS-013</t>
+  </si>
+  <si>
+    <t>High automation supports low crew size and reduces operator workload.</t>
+  </si>
+  <si>
+    <t>Fault-induced throughput degredation</t>
+  </si>
+  <si>
+    <t>System shall prevent uncontrolled termination of production due to single internal component faults.</t>
+  </si>
+  <si>
+    <t>Production coordination</t>
+  </si>
+  <si>
+    <t>System shall coordinate internal operations to satisfy throughput, safety, and logistical constraints concurrently.</t>
+  </si>
+  <si>
+    <t>SN-GS-014</t>
+  </si>
+  <si>
+    <t>SN-GS-015</t>
+  </si>
+  <si>
+    <t>Cooking throughput must not be limited by internal ingredient transport.</t>
+  </si>
+  <si>
+    <t>Ensures the system can transition from inactive to productive operation without extended downtime.</t>
+  </si>
+  <si>
+    <t>Should tolerate individual component failures without complete loss of production.</t>
+  </si>
+  <si>
+    <t>Ensures that throughput, safety, and logistics objectives are met simultaneously in a highly automated system.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -264,7 +447,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -272,322 +455,835 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" customWidth="true"/>
-    <col min="2" max="2" width="21.33203125" customWidth="true"/>
-    <col min="3" max="3" width="92.77734375" customWidth="true"/>
-    <col min="4" max="4" width="89.6640625" customWidth="true"/>
-    <col min="5" max="5" width="11.44140625" customWidth="true"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" customWidth="1"/>
+    <col min="3" max="3" width="92.77734375" customWidth="1"/>
+    <col min="4" max="4" width="89.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>60</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" t="s">
         <v>76</v>
       </c>
     </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>